<commit_message>
Aprimoramento do exercício Back-Scratch
</commit_message>
<xml_diff>
--- a/tabelas/sit_and_reach2.xlsx
+++ b/tabelas/sit_and_reach2.xlsx
@@ -1,3 +1,140 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+</workbook>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
@@ -280,4 +417,339 @@
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Age</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Height</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Weigth</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Real distance</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Calculated distance</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-0.62</v>
+      </c>
+      <c r="G2" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>-24</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-23.51</v>
+      </c>
+      <c r="G3" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6.26</v>
+      </c>
+      <c r="G4" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>-24</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-23.98</v>
+      </c>
+      <c r="G5" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B6" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F6" t="n">
+        <v>4.27</v>
+      </c>
+      <c r="G6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>20</v>
+      </c>
+      <c r="B7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="G7" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>-7</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-7.51</v>
+      </c>
+      <c r="G8" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>20</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>-4</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-4.16</v>
+      </c>
+      <c r="G9" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-1.15</v>
+      </c>
+      <c r="G10" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>20</v>
+      </c>
+      <c r="B11" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-1.28</v>
+      </c>
+      <c r="G11" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>20</v>
+      </c>
+      <c r="B12" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="G12" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>3.05</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Melhorias no Back-Scratch e CS runner
</commit_message>
<xml_diff>
--- a/tabelas/sit_and_reach2.xlsx
+++ b/tabelas/sit_and_reach2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -972,15 +972,11 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>1.74</t>
-        </is>
+      <c r="A24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1.74</v>
       </c>
       <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
@@ -991,14 +987,110 @@
       <c r="E24" t="n">
         <v>-16</v>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>-17.00</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>82</t>
+      <c r="F24" t="n">
+        <v>-17</v>
+      </c>
+      <c r="G24" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="F25" t="n">
+        <v>-13.26</v>
+      </c>
+      <c r="G25" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>20</v>
+      </c>
+      <c r="B26" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>-15.8</v>
+      </c>
+      <c r="F26" t="n">
+        <v>-16.75</v>
+      </c>
+      <c r="G26" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>-16</v>
+      </c>
+      <c r="F27" t="n">
+        <v>-16.44</v>
+      </c>
+      <c r="G27" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1.64</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Feminine</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>-14.2</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>-15.01</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>52</t>
         </is>
       </c>
     </row>

</xml_diff>